<commit_message>
add hyperlink in my_jobs and all job postings to allow users to directly go to linkedin or indeed
</commit_message>
<xml_diff>
--- a/iTrack/scraped_jobs.xlsx
+++ b/iTrack/scraped_jobs.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH12"/>
+  <dimension ref="A1:AH27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,39 +607,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>li-4346667822</t>
+          <t>in-225d4b3b461348b2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4346667822</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>https://ph.indeed.com/viewjob?jk=225d4b3b461348b2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://intrepid.bamboohr.com/careers/1521?source=indeed&amp;src=indeed&amp;postedDate=2026-01-11</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tech Svc Desk - L1</t>
+          <t>Finance Intern (Required Internship Only)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Unisys</t>
+          <t>Intrepid</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Manila, National Capital Region, Philippines</t>
+          <t>Manila, P00, PH</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46022</v>
-      </c>
-      <c r="I2" t="inlineStr"/>
+        <v>46033</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
@@ -652,11 +660,53 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>**Who we are**
+Intrepid Asia is a leading Ecommerce and Digital Solutions Provider in South East Asia. We offer end\-to\-end omni\-channel ecommerce management, Livestreaming, Video production \&amp; Affiliate Management for Social Commerce plus full funnel Digital Marketing Services and advanced Market Intelligence, all powered by state of the art inhouse Technology to our client base of leading international brands across all key marketplaces and social platforms in all 6 SEA countries. Brands love our regional presence, our excellent data\-driven and growth\-focused services which are enabled by the strongest team in the industry, and our advanced marketing and tech capabilities.
+We are growing rapidly and as the exclusive partner of Flywheel in SEA, we offer many exciting opportunities to work with leading brands across multiple categories and key industry players. By joining us, you will work on the cutting edge of digital and social commerce in SEA, and experience what it takes to drive a successful ecommerce business end\-to\-end.
+ **The team you will be part of**
+Our Finance Team is at the core of every major decision we make. We don’t just keep the books — we shape the direction of the business. By delivering on financial insights, strategic analysis, and data\-driven recommendations, the team plays a critical role in guiding growth and ensuring long\-term success. From planning and forecasting to optimizing performance and supporting key commercial initiatives, Our Finance team is a key partner across every function. With a strong focus on integrity, accuracy, and collaboration, its goal is to ensure the company remains financially strong, agile, and ready for the future.
+ **The part you will play**
+We are looking for a Finance Intern who will be an active contributor to our Finance team. This role will report directly to the Senior Accountant and will provide hands\-on exposure to day\-to\-day finance operations, including accounting support, documentation, and financial administrative tasks. You will work closely with the Finance team and gain practical experience in a fast\-paced ecommerce environment.
+ **As a Finance Intern, you will take charge of**
+* Assisting in the preparation and issuance of retail sales invoices
+* Filing, organizing, and maintaining accounting and finance documents
+* Supporting liquidation, reimbursement, and expense claims processes
+* Assisting in accounts receivable and accounts payable tracking
+* Helping ensure completeness and accuracy of financial records
+* Supporting month\-end and ad\-hoc finance reporting tasks
+* Coordinating with internal teams regarding finance\-related documentation
+* Performing other administrative and operational finance tasks as assigned
+**What we are looking for \- the ideal profile**
+* Currently pursuing a Bachelor’s degree in Finance, Accounting, Management Accounting, Business Administration, or a related course
+* Internship **must be a required internship** as part of the university curriculum
+* Able to commit for the full required internship period (minimum duration as required by school)
+* Basic understanding of accounting and finance principles
+* Proficient in Microsoft Suite and Google Workspace
+* Strong attention to detail and good organizational skills
+* Able to handle confidential financial information with integrity
+* Willing to learn, proactive, and able to work in a team environment
+**In return, you will be getting**
+* Join an all\-star Finance team which continues to raise the bar, with systems and processes (and company stability) at the level of sophistication of a small multinational, but with a 'start\-up' spirit of innovation and continuous improvement in an ever\-evolving world
+* In terms of learning opportunities, our organization is second to none. You will get to work on a variety of business models across many different clients as if we are 5 companies in one, and everyone is involved in projects to drive further improvement.
+* Regional teams and country Finance teams collaborate closely to ensure all finance aspects of our business are optimized, giving you a wide exposure and enhanced learning curve in a close\-knit and supportive team
+**We also offer**
+**Best of Both Worlds**
+We are a scale up: the sophistication of a small multinational, with the agility of a start\-up. This means you get to work on cutting\-edge projects, and besides your 'standard' job description, we love to see you show entrepreneurial initiative and want to see your take on how you can take your role and our company to the next level. Good ideas get implemented. You are the master of your own destiny.
+ **Culture that Brings Out the Best**
+At Intrepid, culture is not just a buzzword, it is what we practice at work every day. We believe in collaboration over competition, transparency over politics, and willingness to learn over ego. You will be part of a team where people genuinely support one another, celebrate wins together, and face challenges head\-on as one. We put our all into the work but we balance it with fun, whether that is through team lunches, after\-work hangouts, events or shared laughter in the office. This is a place where you can thrive professionally while having a great time.
+ **Grow Without Limits**
+Learning at Intrepid is constant and dynamic. You will have access to formal training through face\-to\-face sessions, coaching and our very own Intrepid Academy. On top of that, real\-world experience such as leading clients, working with advanced tech, and mastering best\-in\-class processes will accelerate your growth every step of the way. Surrounded by a talented team that raises the bar daily, in a rapidly growing and ever\-expanding business, the opportunities for your development are endless.
+ **Rewarding You Right**
+We believe great work deserves great rewards at Intrepid. That’s why we offer competitive compensation and generous benefits, including comprehensive insurance and ample leave, to support you both in and out of the workplace. We want you to feel valued, cared for, and empowered to bring your best self to work every day.
+ *Note: We will not be accepting any unsolicited resumes or CVs from headhunting or recruitment agencies at this point. Any CVs or profiles shared with us will not be entertained, and in the event of dispute, Intrepid will not be liable for any material compensation to third parties*</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/unisys</t>
+          <t>https://ph.indeed.com/cmp/Intrepid-1c14aa57</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
@@ -675,39 +725,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>li-4346725522</t>
+          <t>in-2dbb6c5d669cc55a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4346725522</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>https://ph.indeed.com/viewjob?jk=2dbb6c5d669cc55a</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://intrepid.bamboohr.com/careers/1520?source=indeed&amp;src=indeed&amp;postedDate=2026-01-11</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Evening Cleaning Tech</t>
+          <t>Human Resources Intern (Required Internship Only)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Office Pride Franchise Opportunity</t>
+          <t>Intrepid</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
+          <t>Manila, P00, PH</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>46022</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
+        <v>46033</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
@@ -720,11 +778,53 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>**Who we are**
+Intrepid Asia is a leading Ecommerce and Digital Solutions Provider in South East Asia. We offer end\-to\-end omni\-channel ecommerce management, Livestreaming, Video production \&amp; Affiliate Management for Social Commerce plus full funnel Digital Marketing Services and advanced Market Intelligence, all powered by state of the art inhouse Technology to our client base of leading international brands across all key marketplaces and social platforms in all 6 SEA countries. Brands love our regional presence, our excellent data\-driven and growth\-focused services which are enabled by the strongest team in the industry, and our advanced marketing and tech capabilities.
+We are growing rapidly and as the exclusive partner of Flywheel in SEA, we offer many exciting opportunities to work with leading brands across multiple categories and key industry players. By joining us, you will work on the cutting edge of digital and social commerce in SEA, and experience what it takes to drive a successful ecommerce business end\-to\-end.
+ **The team you will be part of**
+Our Talent \&amp; People Team is the heartbeat of our organization \- championing a culture where people thrive and potential is unlocked. From attracting top talent and shaping employee experiences to driving development, engagement, and retention, the team plays a strategic role in building and maintaining a high\-performing, empowered workforce. We are here to grow with the business and for the people behind it.
+ **The part you will play**
+We are looking for a Human Resources Intern who will be an active contributor to our People Operations team. This role will report directly to our People Operations Specialist and will provide hands\-on exposure to various HR functions, supporting daily operations and ongoing initiatives.
+ **As an HR Intern, you will take charge of**
+* Assisting in preparing orientation materials and schedules for new employees
+* Helping maintain employee records and ensure confidentiality
+* Supporting the resolution of employee queries and concerns
+* Assisting in organizing employee engagement activities and events
+* Assisting in maintaining and updating HR 201 files and database
+* Assisting in the preparation of HR\-related reports and documents as needed
+* Assisting in coordinating training sessions and workshops
+* Participating in the development of training materials
+* Providing general administrative support to the HR department
+* Participating in HR projects and initiatives as assigned
+**What we are looking for \- the ideal profile**
+* Currently pursuing a degree in Human Resource Management, Psychology, or other related fields, **with an internship requirement**
+* Strong written and verbal communication skills
+* Proficient in MS Office applications and Google Workspace
+* Detail\-oriented with the ability to handle sensitive and confidential information
+* Strong organizational skills with the ability to manage multiple tasks and meet deadlines
+**In return, you will be getting**
+* Tackling the sophisticated people's challenges in the rapidly evolving e\-commerce landscape with data insights and innovative solutions.
+* You will be joining an all\-star People Team that consistently raises the bar by combining the systems and processes of a small multinational with the collaborative, innovative, and agile spirit of a startup in an ever\-evolving world.
+* With our team’s rapid growth and the People Team launching new initiatives to enhance both employee experience and performance, you will benefit from a wide range of opportunities for development. Our structured learning programs covering both functional skills and broader growth are designed to support you at every stage of your journey
+* Our supportive culture and close collaboration between regional and local teams create a close\-knit work environment which many in our team love and thrive in
+**We also offer**
+**Best of Both Worlds**
+We are a scale up: the sophistication of a small multinational, with the agility of a start\-up. This means you get to work on cutting\-edge projects, and besides your 'standard' job description, we love to see you show entrepreneurial initiative and want to see your take on how you can take your role and our company to the next level. Good ideas get implemented. You are the master of your own destiny.
+ **Culture that Brings Out the Best**
+At Intrepid, culture is not just a buzzword, it is what we practice at work every day. We believe in collaboration over competition, transparency over politics, and willingness to learn over ego. You will be part of a team where people genuinely support one another, celebrate wins together, and face challenges head\-on as one. We put our all into the work but we balance it with fun, whether that is through team lunches, after\-work hangouts, events or shared laughter in the office. This is a place where you can thrive professionally while having a great time.
+ **Grow Without Limits**
+Learning at Intrepid is constant and dynamic. You will have access to formal training through face\-to\-face sessions, coaching and our very own Intrepid Academy. On top of that, real\-world experience such as leading clients, working with advanced tech, and mastering best\-in\-class processes will accelerate your growth every step of the way. Surrounded by a talented team that raises the bar daily, in a rapidly growing and ever\-expanding business, the opportunities for your development are endless.
+ **Rewarding You Right**
+We believe great work deserves great rewards at Intrepid. That’s why we offer competitive compensation and generous benefits, including comprehensive insurance and ample leave, to support you both in and out of the workplace. We want you to feel valued, cared for, and empowered to bring your best self to work every day.
+ *Note: We will not be accepting any unsolicited resumes or CVs from headhunting or recruitment agencies at this point. Any CVs or profiles shared with us will not be entertained, and in the event of dispute, Intrepid will not be liable for any material compensation to third parties*</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/office-pride-franchise-opportunity</t>
+          <t>https://ph.indeed.com/cmp/Intrepid-1c14aa57</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
@@ -743,39 +843,47 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>li-4308717661</t>
+          <t>in-f1e13e490a93b540</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4308717661</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>https://ph.indeed.com/viewjob?jk=f1e13e490a93b540</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/it-programming-intern-f1e13e490a93b540</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Technician</t>
+          <t>IT / Programming Intern</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Konecranes</t>
+          <t>Lucky Boba</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pampanga, Central Luzon, Philippines</t>
+          <t>Sangandaan, P00, PH</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>46022</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>46032</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>temporary, internship</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
@@ -787,12 +895,54 @@
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>luckyboba.hr@gmail.com</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>**We're Hiring Interns!**
+Are you passionate about technology and eager to gain  
+hands\-on experience in IT and programming? Join our team and kickstart your  
+career!
+**Position:** IT / Programming Intern
+**Who We’re Looking For:**  
+**Students currently pursuing:**
+IT Programming  
+Computer Engineering  
+Computer Science  
+Any Programming\-related course
+**What You’ll Do:**  
+Assist in software development and coding projects  
+Support IT operations and system maintenance  
+Collaborate with our tech team on real\-world projects  
+Learn best practices in programming, debugging, and testing
+**What We’re Looking For:**  
+Strong interest in programming and technology  
+Basic knowledge of programming languages (e.g., Java, Python, C\#, or JavaScript)  
+Eagerness to learn and take on challenges  
+Good communication and teamwork skills
+**Perks \&amp; Benefits:**  
+Hands\-on experience in real projects  
+Mentorship from experienced developers  
+Flexible working hours  
+Certificate of Internship upon completion
+**How to Apply:**  
+Submit your CV \&amp; Portfolio**: luckyboba.hr@gmail.com**
+Start your tech journey with us!
+Job Types: Temporary, OJT (On the job training)  
+Contract length: 3 months
+Benefits:
+* Flexible schedule
+* Flextime
+Work Location: In person</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>https://fi.linkedin.com/company/konecranes</t>
+          <t>https://ph.indeed.com/cmp/Lucky-Boba-1</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
@@ -811,39 +961,47 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>li-4329605575</t>
+          <t>in-87c8416ce707a201</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4329605575</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>https://ph.indeed.com/viewjob?jk=87c8416ce707a201</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/business-development-intern-paid-ojt-87c8416ce707a201</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Reefer Technician</t>
+          <t>Business Development Intern (Paid OJT)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>IRS Eastern, Inc.</t>
+          <t>Achieve Without Borders, Inc. (AWB)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Malabon, National Capital Region, Philippines</t>
+          <t>Makati, P00, PH</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>46021</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
+        <v>46032</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -856,16 +1014,63 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>**About the Role:**  
+If you’ve ever wanted to learn how to charm clients, close deals, and sound smart while doing it, this one’s for you. Achieve Without Borders, Inc. (AWB) is opening its doors to aspiring sales superheroes who are ready to roll up their sleeves, dive into the business world, and make things happen with free lunch to fuel the hustle.
+**What You’ll Be Doing:**
+* Help our sales team turn leads into happy clients (and happy clients into loyal ones).
+* Assist in making presentations that wow, not zzz.
+* Keep our CRM up to date because organized data equals world domination.
+* Join team huddles, pitch your ideas, and learn the fine art of selling without sounding salesy.
+* Track leads, send follow\-ups, and help us build relationships that last longer than most New Year’s resolutions.
+**Who You Are:**
+* A student in Business, Marketing, or Communications (or someone who just loves making connections).
+* Confident, proactive, and just the right amount of persuasive.
+* Knows how to use Microsoft Office (and maybe even CRM tools if you’re feeling fancy).
+* Detail\-oriented and professional, even when you’re having fun.
+* **Makati bound.**
+**Why Join AWB?**
+* Real\-world experience with mentors who’ve been there, sold that.
+* Paid training and free meals because good ideas need fuel.
+* A chance to grow your career in tech\-driven business development.
+* **Perform well, and we might just hire you for real.**
+**ABOUT ACHIEVE WITHOUT BORDERS (AWB)** 
+Achieve Without Borders Inc. (AWB) is a Philippine\-based IT solutions company headquartered in Makati City. We are a **Gold Odoo Partner and Google Partner**, dedicated to helping Filipino businesses streamline operations and scale through ERP, cloud, and digital transformation solutions.
+Our expertise spans ERP systems (Odoo, NetSuite), cloud platforms (Google Cloud), and enterprise productivity tools (Microsoft 365, Google Workspace). We combine business insight and technology to deliver smart, integrated systems that empower organizations to work smarter and grow faster.
+Job Type: OJT (On the job training)  
+Contract length: 3 months
+Benefits:
+* Paid training
+* Promotion to permanent employee
+* Staff meals provided
+Work Location: In person</t>
+        </is>
+      </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://ph.linkedin.com/company/irs-eastern-inc</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+          <t>https://ph.indeed.com/cmp/Achieve-Without-Borders,-Inc.-(awb)</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>https://d2q79iu7y748jz.cloudfront.net/s/_squarelogo/256x256/5108215db8072827f110d419c3f8313d</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>https://www.achievewithoutborders.com</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>2029 Gen Mascardo Street
+    Barangay Bangkal
+    Makati City MM
+    Philippines</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
@@ -879,39 +1084,47 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>li-4340991467</t>
+          <t>in-b20557a09f0fdf0f</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4340991467</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>https://ph.indeed.com/viewjob?jk=b20557a09f0fdf0f</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/sales-and-marketing-intern-paid-ojt-b20557a09f0fdf0f</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Tech Coord, Fund Acctng</t>
+          <t>Sales and Marketing Intern (Paid OJT)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Northern Trust</t>
+          <t>Achieve Without Borders, Inc. (AWB)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Manila, National Capital Region, Philippines</t>
+          <t>Makati, P00, PH</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46021</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
+        <v>46032</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
@@ -924,16 +1137,67 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>**Be the Hype Behind the Tech**
+Can you sell sand in a desert, or at least convince your friends to join your group project?  
+Do you scroll through ads and think, "*I could totally write something better*"?  
+If so, Achieve Without Borders Inc. (AWB) wants you on our team as our next **Sales and Marketing Intern.**
+We are a Gold Odoo Partner, Google Partner, and an all\-around IT wizard squad that helps businesses modernize through ERP, Cloud, and Network Solutions. Translation: we make companies smarter, faster, and slightly cooler.
+Now, we need creative minds who can tell that story to the world.
+**What You’ll Be Doing (a.k.a. How You’ll Look Busy on LinkedIn)**
+* Cook up digital marketing campaigns that actually make people stop scrolling.
+* Turn coffee and creativity into engaging social media content, blogs, and visuals.
+* Help launch webinars, events, and promos that make our brand shine brighter than your screen’s blue light.
+* Research market trends like a detective with Wi\-Fi.
+* Join sales and marketing projects that connect our tech magic to real business growth.
+* Collaborate with awesome people (yes, we’re biased).
+**What We’re Looking For**
+* Currently taking up Marketing, Business, Communications, or something equally awesome.
+* Fluent in English, creativity, and Google Workspace.
+* Knows a thing or two about social media marketing, content creation, and branding.
+* Canva or Adobe familiarity equals instant brownie points.
+* Organized, proactive, and allergic to boredom.
+* **Can join us onsite in Makati City.**
+**What’s In It For You**
+* Real\-world experience in digital marketing, sales strategy, and tech branding.
+* Mentorship from professionals who actually care about your growth.
+* Exposure to ERP, cloud, and network technologies (a.k.a. resume gold).
+* **Paid training and free daily lunch (yes, free).**
+* A shot at becoming part of the AWB family after your internship.
+Job Type: OJT (On the job training)  
+Contract length: 3 months
+Benefits:
+* Paid training
+* Promotion to permanent employee
+* Staff meals provided
+Work Location: In person</t>
+        </is>
+      </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/northern-trust</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+          <t>https://ph.indeed.com/cmp/Achieve-Without-Borders,-Inc.-(awb)</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>https://d2q79iu7y748jz.cloudfront.net/s/_squarelogo/256x256/5108215db8072827f110d419c3f8313d</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>https://www.achievewithoutborders.com</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>2029 Gen Mascardo Street
+    Barangay Bangkal
+    Makati City MM
+    Philippines</t>
+        </is>
+      </c>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
@@ -947,56 +1211,104 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>li-4336353053</t>
+          <t>in-14ad7cd35cfbb3dc</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4336353053</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>https://ph.indeed.com/viewjob?jk=14ad7cd35cfbb3dc</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/business-development-intern-14ad7cd35cfbb3dc</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Service Technical Support IX</t>
+          <t>Business Development Intern</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>Founders Launchpad</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Mandaluyong, National Capital Region, Philippines</t>
+          <t>Makati, P00, PH</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46021</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
+        <v>46031</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>parttime, internship</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>**Job Summary**
+As an **Analyst Intern**, you will work hands\-on with one of our ventures to drive growth through sales pipeline development, GTM strategy execution, and strategic partnerships—taking a founder's mindset while supporting operational initiatives and growth experiments in a fast\-paced startup environment.
+**Job Responsibilities**
+**Business Development for a Venture**
+* **Market Expansion:** Support sales pipeline building, customer outreach, and partnerships for one of our ventures.
+* **Go\-to\-Market Execution:** Assist in building and executing GTM strategies, including messaging, materials, CRM management, and lead generation.
+* **Growth Experiments:** Test and analyze marketing, sales, and operational experiments to help scale the venture.
+* **Operations Support:** Collaborate with the venture’s founders on internal tools, process design, and strategic projects as needed.
+**Qualifications**
+* Currently enrolled in a Bachelor's degree program, preferably in their third or fourth year, with a focus on Business, Finance, Economics, or a related field.
+* Prior internship experience or relevant coursework is a plus, but not required.
+* Strong analytical skills with the ability to break down problems and use data to drive decisions.
+* Proven initiative and comfort with ambiguity — you are resourceful, solutions\-driven, and thrive in fast\-paced environments.
+* Deep curiosity about startups, innovation, and building from 0 to 1\.
+* Excellent written and verbal communication skills.
+* A hands\-on, founder\-like mentality — you’re not afraid to take ownership.
+* Available to commit to a minimum 3\-month internship, with potential for extension into a long\-term internship or full\-time opportunity.
+**Bonus Points**
+* Familiarity with tools like Notion, Airtable, Monday.com, Hubspot, or SQL.
+* Prior startup experience.
+* Passion for a specific domain such as fintech, logistics, healthtech, or consumer tech.
+**Why Work with Us?**
+* Work with a young, passionate, and fun team
+* We offer a diverse and international work environment
+* Hybrid exposure to venture capital and startup building — unique experience for future founders or operators.
+* Mentorship from experienced founders and operators.
+* A high\-growth environment with ownership and learning from day one.
+Job Types: Part\-time, OJT (On the job training), Fresh graduate  
+Contract length: 3 months
+Pay: Php5,000\.00 \- Php10,000\.00 per month
+Expected hours: 30 – 40 per week
+Benefits:
+* Flexible schedule
+* Flextime
+* Paid training
+* Work from home
+Work Location: In person</t>
+        </is>
+      </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/vertiv</t>
+          <t>https://ph.indeed.com/cmp/Founders-Launchpad</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1015,7 +1327,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>li-4326334571</t>
+          <t>li-4345212547</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1025,27 +1337,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4326334571</t>
+          <t>https://www.linkedin.com/jobs/view/4345212547</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>On Site Service Technician - Level I</t>
+          <t>Deskside Technician</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Cummins Asia Pacific</t>
+          <t>Stefanini North America and APAC</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Laguna, Calabarzon, Philippines</t>
+          <t>Pasay, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46021</v>
+        <v>46032</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1064,7 +1376,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://au.linkedin.com/company/cummins-asiapacific</t>
+          <t>https://br.linkedin.com/company/stefanini-na-apac</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1083,7 +1395,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4336403679</t>
+          <t>li-4334598816</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1093,27 +1405,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4336403679</t>
+          <t>https://www.linkedin.com/jobs/view/4334598816</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Technician, Reliability</t>
+          <t>Service Technician Castilla y León</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Allegro MicroSystems</t>
+          <t>Vestas</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>National Capital Region, Philippines</t>
+          <t>Buenavista, Western Visayas, Philippines</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46021</v>
+        <v>46032</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -1132,7 +1444,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/allegro-microsystems</t>
+          <t>https://dk.linkedin.com/company/vestas</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1151,7 +1463,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4329620923</t>
+          <t>li-4350286936</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1161,18 +1473,18 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4329620923</t>
+          <t>https://www.linkedin.com/jobs/view/4350286936</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Air Condition Technician</t>
+          <t>Technician I, Managed Sevices</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Ardenhills Suites Corporation</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1181,7 +1493,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46020</v>
+        <v>46032</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1200,7 +1512,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://ph.linkedin.com/company/ardenhillssuites</t>
+          <t>https://www.linkedin.com/company/copeland</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1219,7 +1531,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4336896543</t>
+          <t>li-4350237071</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1229,26 +1541,28 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4336896543</t>
+          <t>https://www.linkedin.com/jobs/view/4350237071</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Back-end Technical Lead</t>
+          <t>Technician I, Managed Services</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Cebu Pacific Air</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pasay, National Capital Region, Philippines</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>Quezon City, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>46032</v>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -1266,7 +1580,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://ph.linkedin.com/company/cebupacificair</t>
+          <t>https://www.linkedin.com/company/copeland</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1285,7 +1599,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4346786201</t>
+          <t>li-4350187030</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1295,22 +1609,28 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4346786201</t>
+          <t>https://www.linkedin.com/jobs/view/4350187030</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Japanese Tech Bilingual – Java Spring Boot</t>
+          <t>Technician I, Managed Services</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>PROTALENTNEXUS CONSULTING</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+          <t>Copeland</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Quezon City, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>46032</v>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -1328,7 +1648,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://ng.linkedin.com/company/protalentnexus</t>
+          <t>https://www.linkedin.com/company/copeland</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1344,6 +1664,1012 @@
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr"/>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>li-4359465790</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4359465790</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Platform Technician I</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>BlueVoyant</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Manila, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="b">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/bluevoyant</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>li-4332222982</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4332222982</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Technical Services Technician</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Datumstruct Philippines, Inc.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Makati, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="b">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>https://ph.linkedin.com/company/datumstructph</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>li-4314154195</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4314154195</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026 Data Center Technician Intern</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Amazon Web Services (AWS)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Bolinao, Ilocos Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="b">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/amazon-web-services</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>li-4331574126</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4331574126</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Multi-Skilled Technician - Makati</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CBRE Asia Pacific</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Makati, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="b">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>li-4352057410</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4352057410</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Associate, Technical Services</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Vena Group</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Ilocos Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="b">
+        <v>0</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>https://sg.linkedin.com/company/venagroup</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>li-4359761815</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4359761815</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Technician I - Reliability</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Microchip Technology Inc.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Davao, Davao Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="b">
+        <v>0</v>
+      </c>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/microchip-technology</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>li-4359761816</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4359761816</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Technician I - Reliability</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Microchip Technology Inc.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Davao, Davao Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="b">
+        <v>0</v>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/microchip-technology</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>li-4359611660</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4359611660</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Multi-Skilled Technician</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>JLL</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Makati, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>46031</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="b">
+        <v>0</v>
+      </c>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/jll</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>li-4358913747</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4358913747</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Tech Svc Desk</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Unisys</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Manila, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>46030</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="b">
+        <v>0</v>
+      </c>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/unisys</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>li-4358576241</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4358576241</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sr Tech Svc Desk</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Unisys</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Manila, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>46030</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="b">
+        <v>0</v>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/unisys</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>li-4359757191</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4359757191</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Medewerker Technische Dienst</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Stayokay</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Bacnotan, Ilocos Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="b">
+        <v>0</v>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>https://nl.linkedin.com/company/stayokay</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>li-4359964843</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4359964843</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Multi Skilled Technician</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>JLL</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Makati, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="b">
+        <v>0</v>
+      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/jll</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>li-4345800265</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4345800265</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SRE Technician</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>STMicroelectronics</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Calamba, Northern Mindanao, Philippines</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="b">
+        <v>0</v>
+      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>https://ch.linkedin.com/company/stmicroelectronics</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>li-4334726725</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4334726725</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Renewables Technical Lead</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="b">
+        <v>0</v>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>https://uk.linkedin.com/company/aggreko</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>li-4360643379</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4360643379</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Multi Skilled Technician</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>JLL</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Batangas, Calabarzon, Philippines</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="b">
+        <v>0</v>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/jll</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add activity model to allow dashboard to display recent activity
</commit_message>
<xml_diff>
--- a/iTrack/scraped_jobs.xlsx
+++ b/iTrack/scraped_jobs.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH27"/>
+  <dimension ref="A1:AH25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,7 +607,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>in-225d4b3b461348b2</t>
+          <t>in-a0f2177ec4d1d3ea</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -617,31 +617,31 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://ph.indeed.com/viewjob?jk=225d4b3b461348b2</t>
+          <t>https://ph.indeed.com/viewjob?jk=a0f2177ec4d1d3ea</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://intrepid.bamboohr.com/careers/1521?source=indeed&amp;src=indeed&amp;postedDate=2026-01-11</t>
+          <t>http://ph.indeed.com/job/accounting-intern-a0f2177ec4d1d3ea</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Finance Intern (Required Internship Only)</t>
+          <t>Accounting Intern</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Intrepid</t>
+          <t>Agile Tech Ops Ince</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Manila, P00, PH</t>
+          <t>Ayala Avenue-Paseo de Roxas, P00, PH</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46033</v>
+        <v>46035</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -661,6 +661,113 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
+        <is>
+          <t>**JOB TITLE:** Accounting Intern
+**COMPANY:** Agile Tech Ops Inc.
+**LOCATION:** Makati (On\-site / Hybrid)
+**INTERNSHIP TYPE:** Internship / OJT
+**JOB SUMMARY**  
+Agile Tech Ops Inc. is seeking a motivated and detail\-oriented **Accounting Intern** to support our Finance and Accounting team. This internship provides hands\-on experience in basic accounting processes, financial documentation, and office operations while working closely with experienced professionals.
+**KEY RESPONSIBILITIES**  
+Assist in preparing, encoding, and maintaining accounting records and documents
+Support accounts payable and receivable monitoring
+Organize invoices, receipts, vouchers, and other financial files
+Assist in bank reconciliations and expense tracking
+Provide support during audits and month\-end reporting
+Perform other accounting and administrative tasks as assigned
+**QUALIFICATIONS**
+Currently taking **BS Accountancy, BS Accounting Technology, or any Finance\-related course**
+Must be endorsed by school for internship / OJT
+Basic knowledge of accounting principles is an advantage
+Proficient in MS Excel and MS Word
+Detail\-oriented, organized, and willing to learn
+Able to work independently and meet deadlines
+**WHAT WE OFFER**
+Hands\-on accounting experience in a corporate setting
+Mentorship from experienced accounting professionals
+Internship allowance (if applicable)
+Certificate of Completion upon successful internship
+Opportunity for future employment based on performance
+Job Type: OJT (On the job training)
+Work Location: In person</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/cmp/Agile-Tech-Ops-Ince</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>in-225d4b3b461348b2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/viewjob?jk=225d4b3b461348b2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://intrepid.bamboohr.com/careers/1521?source=indeed&amp;src=indeed&amp;postedDate=2026-01-11</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Finance Intern (Required Internship Only)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Intrepid</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Manila, P00, PH</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>46033</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
         <is>
           <t>**Who we are**
 Intrepid Asia is a leading Ecommerce and Digital Solutions Provider in South East Asia. We offer end\-to\-end omni\-channel ecommerce management, Livestreaming, Video production \&amp; Affiliate Management for Social Commerce plus full funnel Digital Marketing Services and advanced Market Intelligence, all powered by state of the art inhouse Technology to our client base of leading international brands across all key marketplaces and social platforms in all 6 SEA countries. Brands love our regional presence, our excellent data\-driven and growth\-focused services which are enabled by the strongest team in the industry, and our advanced marketing and tech capabilities.
@@ -703,82 +810,82 @@
  *Note: We will not be accepting any unsolicited resumes or CVs from headhunting or recruitment agencies at this point. Any CVs or profiles shared with us will not be entertained, and in the event of dispute, Intrepid will not be liable for any material compensation to third parties*</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
         <is>
           <t>https://ph.indeed.com/cmp/Intrepid-1c14aa57</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>in-2dbb6c5d669cc55a</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>indeed</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>https://ph.indeed.com/viewjob?jk=2dbb6c5d669cc55a</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>https://intrepid.bamboohr.com/careers/1520?source=indeed&amp;src=indeed&amp;postedDate=2026-01-11</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Human Resources Intern (Required Internship Only)</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Intrepid</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Manila, P00, PH</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>46033</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>internship</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="b">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="b">
         <v>0</v>
       </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
         <is>
           <t>**Who we are**
 Intrepid Asia is a leading Ecommerce and Digital Solutions Provider in South East Asia. We offer end\-to\-end omni\-channel ecommerce management, Livestreaming, Video production \&amp; Affiliate Management for Social Commerce plus full funnel Digital Marketing Services and advanced Market Intelligence, all powered by state of the art inhouse Technology to our client base of leading international brands across all key marketplaces and social platforms in all 6 SEA countries. Brands love our regional presence, our excellent data\-driven and growth\-focused services which are enabled by the strongest team in the industry, and our advanced marketing and tech capabilities.
@@ -821,86 +928,86 @@
  *Note: We will not be accepting any unsolicited resumes or CVs from headhunting or recruitment agencies at this point. Any CVs or profiles shared with us will not be entertained, and in the event of dispute, Intrepid will not be liable for any material compensation to third parties*</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
         <is>
           <t>https://ph.indeed.com/cmp/Intrepid-1c14aa57</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>in-f1e13e490a93b540</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>indeed</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>https://ph.indeed.com/viewjob?jk=f1e13e490a93b540</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>http://ph.indeed.com/job/it-programming-intern-f1e13e490a93b540</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>IT / Programming Intern</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Lucky Boba</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Sangandaan, P00, PH</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>46032</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>temporary, internship</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="b">
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="b">
         <v>0</v>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
         <is>
           <t>luckyboba.hr@gmail.com</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>**We're Hiring Interns!**
 Are you passionate about technology and eager to gain  
@@ -939,138 +1046,15 @@
 Work Location: In person</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/cmp/Lucky-Boba-1</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>in-87c8416ce707a201</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/viewjob?jk=87c8416ce707a201</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>http://ph.indeed.com/job/business-development-intern-paid-ojt-87c8416ce707a201</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Business Development Intern (Paid OJT)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Achieve Without Borders, Inc. (AWB)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Makati, P00, PH</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>46032</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>internship</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>**About the Role:**  
-If you’ve ever wanted to learn how to charm clients, close deals, and sound smart while doing it, this one’s for you. Achieve Without Borders, Inc. (AWB) is opening its doors to aspiring sales superheroes who are ready to roll up their sleeves, dive into the business world, and make things happen with free lunch to fuel the hustle.
-**What You’ll Be Doing:**
-* Help our sales team turn leads into happy clients (and happy clients into loyal ones).
-* Assist in making presentations that wow, not zzz.
-* Keep our CRM up to date because organized data equals world domination.
-* Join team huddles, pitch your ideas, and learn the fine art of selling without sounding salesy.
-* Track leads, send follow\-ups, and help us build relationships that last longer than most New Year’s resolutions.
-**Who You Are:**
-* A student in Business, Marketing, or Communications (or someone who just loves making connections).
-* Confident, proactive, and just the right amount of persuasive.
-* Knows how to use Microsoft Office (and maybe even CRM tools if you’re feeling fancy).
-* Detail\-oriented and professional, even when you’re having fun.
-* **Makati bound.**
-**Why Join AWB?**
-* Real\-world experience with mentors who’ve been there, sold that.
-* Paid training and free meals because good ideas need fuel.
-* A chance to grow your career in tech\-driven business development.
-* **Perform well, and we might just hire you for real.**
-**ABOUT ACHIEVE WITHOUT BORDERS (AWB)** 
-Achieve Without Borders Inc. (AWB) is a Philippine\-based IT solutions company headquartered in Makati City. We are a **Gold Odoo Partner and Google Partner**, dedicated to helping Filipino businesses streamline operations and scale through ERP, cloud, and digital transformation solutions.
-Our expertise spans ERP systems (Odoo, NetSuite), cloud platforms (Google Cloud), and enterprise productivity tools (Microsoft 365, Google Workspace). We combine business insight and technology to deliver smart, integrated systems that empower organizations to work smarter and grow faster.
-Job Type: OJT (On the job training)  
-Contract length: 3 months
-Benefits:
-* Paid training
-* Promotion to permanent employee
-* Staff meals provided
-Work Location: In person</t>
-        </is>
-      </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>https://ph.indeed.com/cmp/Achieve-Without-Borders,-Inc.-(awb)</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>https://d2q79iu7y748jz.cloudfront.net/s/_squarelogo/256x256/5108215db8072827f110d419c3f8313d</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>https://www.achievewithoutborders.com</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>2029 Gen Mascardo Street
-    Barangay Bangkal
-    Makati City MM
-    Philippines</t>
-        </is>
-      </c>
+          <t>https://ph.indeed.com/cmp/Lucky-Boba-1</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
@@ -1084,47 +1068,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>in-b20557a09f0fdf0f</t>
+          <t>li-4332535951</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://ph.indeed.com/viewjob?jk=b20557a09f0fdf0f</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>http://ph.indeed.com/job/sales-and-marketing-intern-paid-ojt-b20557a09f0fdf0f</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4332535951</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sales and Marketing Intern (Paid OJT)</t>
+          <t>Technician 1 Monitoring Services (Technical Support)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Achieve Without Borders, Inc. (AWB)</t>
+          <t>Risewave Consulting, Inc.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Makati, P00, PH</t>
+          <t>Quezon City, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>46032</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>internship</t>
-        </is>
-      </c>
+        <v>46034</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
@@ -1137,67 +1113,16 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>**Be the Hype Behind the Tech**
-Can you sell sand in a desert, or at least convince your friends to join your group project?  
-Do you scroll through ads and think, "*I could totally write something better*"?  
-If so, Achieve Without Borders Inc. (AWB) wants you on our team as our next **Sales and Marketing Intern.**
-We are a Gold Odoo Partner, Google Partner, and an all\-around IT wizard squad that helps businesses modernize through ERP, Cloud, and Network Solutions. Translation: we make companies smarter, faster, and slightly cooler.
-Now, we need creative minds who can tell that story to the world.
-**What You’ll Be Doing (a.k.a. How You’ll Look Busy on LinkedIn)**
-* Cook up digital marketing campaigns that actually make people stop scrolling.
-* Turn coffee and creativity into engaging social media content, blogs, and visuals.
-* Help launch webinars, events, and promos that make our brand shine brighter than your screen’s blue light.
-* Research market trends like a detective with Wi\-Fi.
-* Join sales and marketing projects that connect our tech magic to real business growth.
-* Collaborate with awesome people (yes, we’re biased).
-**What We’re Looking For**
-* Currently taking up Marketing, Business, Communications, or something equally awesome.
-* Fluent in English, creativity, and Google Workspace.
-* Knows a thing or two about social media marketing, content creation, and branding.
-* Canva or Adobe familiarity equals instant brownie points.
-* Organized, proactive, and allergic to boredom.
-* **Can join us onsite in Makati City.**
-**What’s In It For You**
-* Real\-world experience in digital marketing, sales strategy, and tech branding.
-* Mentorship from professionals who actually care about your growth.
-* Exposure to ERP, cloud, and network technologies (a.k.a. resume gold).
-* **Paid training and free daily lunch (yes, free).**
-* A shot at becoming part of the AWB family after your internship.
-Job Type: OJT (On the job training)  
-Contract length: 3 months
-Benefits:
-* Paid training
-* Promotion to permanent employee
-* Staff meals provided
-Work Location: In person</t>
-        </is>
-      </c>
+      <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>https://ph.indeed.com/cmp/Achieve-Without-Borders,-Inc.-(awb)</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>https://d2q79iu7y748jz.cloudfront.net/s/_squarelogo/256x256/5108215db8072827f110d419c3f8313d</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>https://www.achievewithoutborders.com</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>2029 Gen Mascardo Street
-    Barangay Bangkal
-    Makati City MM
-    Philippines</t>
-        </is>
-      </c>
+          <t>https://ph.linkedin.com/company/risewave-consulting-inc</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
@@ -1211,104 +1136,56 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>in-14ad7cd35cfbb3dc</t>
+          <t>li-4359997663</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://ph.indeed.com/viewjob?jk=14ad7cd35cfbb3dc</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>http://ph.indeed.com/job/business-development-intern-14ad7cd35cfbb3dc</t>
-        </is>
-      </c>
+          <t>https://www.linkedin.com/jobs/view/4359997663</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Business Development Intern</t>
+          <t>Multi Skilled Technician (Taguig)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Founders Launchpad</t>
+          <t>JLL</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Makati, P00, PH</t>
+          <t>Taguig, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>46031</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>parttime, internship</t>
-        </is>
-      </c>
+        <v>46034</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>**Job Summary**
-As an **Analyst Intern**, you will work hands\-on with one of our ventures to drive growth through sales pipeline development, GTM strategy execution, and strategic partnerships—taking a founder's mindset while supporting operational initiatives and growth experiments in a fast\-paced startup environment.
-**Job Responsibilities**
-**Business Development for a Venture**
-* **Market Expansion:** Support sales pipeline building, customer outreach, and partnerships for one of our ventures.
-* **Go\-to\-Market Execution:** Assist in building and executing GTM strategies, including messaging, materials, CRM management, and lead generation.
-* **Growth Experiments:** Test and analyze marketing, sales, and operational experiments to help scale the venture.
-* **Operations Support:** Collaborate with the venture’s founders on internal tools, process design, and strategic projects as needed.
-**Qualifications**
-* Currently enrolled in a Bachelor's degree program, preferably in their third or fourth year, with a focus on Business, Finance, Economics, or a related field.
-* Prior internship experience or relevant coursework is a plus, but not required.
-* Strong analytical skills with the ability to break down problems and use data to drive decisions.
-* Proven initiative and comfort with ambiguity — you are resourceful, solutions\-driven, and thrive in fast\-paced environments.
-* Deep curiosity about startups, innovation, and building from 0 to 1\.
-* Excellent written and verbal communication skills.
-* A hands\-on, founder\-like mentality — you’re not afraid to take ownership.
-* Available to commit to a minimum 3\-month internship, with potential for extension into a long\-term internship or full\-time opportunity.
-**Bonus Points**
-* Familiarity with tools like Notion, Airtable, Monday.com, Hubspot, or SQL.
-* Prior startup experience.
-* Passion for a specific domain such as fintech, logistics, healthtech, or consumer tech.
-**Why Work with Us?**
-* Work with a young, passionate, and fun team
-* We offer a diverse and international work environment
-* Hybrid exposure to venture capital and startup building — unique experience for future founders or operators.
-* Mentorship from experienced founders and operators.
-* A high\-growth environment with ownership and learning from day one.
-Job Types: Part\-time, OJT (On the job training), Fresh graduate  
-Contract length: 3 months
-Pay: Php5,000\.00 \- Php10,000\.00 per month
-Expected hours: 30 – 40 per week
-Benefits:
-* Flexible schedule
-* Flextime
-* Paid training
-* Work from home
-Work Location: In person</t>
-        </is>
-      </c>
+      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>https://ph.indeed.com/cmp/Founders-Launchpad</t>
+          <t>https://www.linkedin.com/company/jll</t>
         </is>
       </c>
       <c r="W7" t="inlineStr"/>
@@ -1327,7 +1204,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>li-4345212547</t>
+          <t>li-4352672394</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1337,27 +1214,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4345212547</t>
+          <t>https://www.linkedin.com/jobs/view/4352672394</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Deskside Technician</t>
+          <t>PHL Senior Technician - L3 - Represented/Tariff</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Stefanini North America and APAC</t>
+          <t>Dow</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pasay, National Capital Region, Philippines</t>
+          <t>Las Piñas, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>46032</v>
+        <v>46034</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1376,7 +1253,7 @@
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://br.linkedin.com/company/stefanini-na-apac</t>
+          <t>https://www.linkedin.com/company/dow-chemical</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1395,7 +1272,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4334598816</t>
+          <t>li-4351866176</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1405,27 +1282,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4334598816</t>
+          <t>https://www.linkedin.com/jobs/view/4351866176</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Service Technician Castilla y León</t>
+          <t>Multi-Skilled Technician -Lipa</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Vestas</t>
+          <t>CBRE Asia Pacific</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Buenavista, Western Visayas, Philippines</t>
+          <t>Lipa, Calabarzon, Philippines</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46032</v>
+        <v>46034</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -1444,7 +1321,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/company/vestas</t>
+          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1463,7 +1340,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4350286936</t>
+          <t>li-4345396142</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1473,27 +1350,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4350286936</t>
+          <t>https://www.linkedin.com/jobs/view/4345396142</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Technician I, Managed Sevices</t>
+          <t>Multi-Skilled Technician - Lipa</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>CBRE Asia Pacific</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
+          <t>Lipa, Calabarzon, Philippines</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46032</v>
+        <v>46034</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1512,7 +1389,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/copeland</t>
+          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1531,7 +1408,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4350237071</t>
+          <t>li-4334726725</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1541,27 +1418,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4350237071</t>
+          <t>https://www.linkedin.com/jobs/view/4334726725</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Technician I, Managed Services</t>
+          <t>Renewables Technical Lead</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Copeland</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
-        </is>
-      </c>
+          <t>Aggreko</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" s="2" t="n">
-        <v>46032</v>
+        <v>46033</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1580,7 +1453,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/copeland</t>
+          <t>https://uk.linkedin.com/company/aggreko</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1599,7 +1472,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4350187030</t>
+          <t>li-4359964843</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1609,27 +1482,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4350187030</t>
+          <t>https://www.linkedin.com/jobs/view/4359964843</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Technician I, Managed Services</t>
+          <t>Multi Skilled Technician</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>JLL</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
+          <t>Makati, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46032</v>
+        <v>46033</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1648,7 +1521,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/copeland</t>
+          <t>https://www.linkedin.com/company/jll</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1667,7 +1540,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>li-4359465790</t>
+          <t>li-4360643379</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1677,27 +1550,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359465790</t>
+          <t>https://www.linkedin.com/jobs/view/4360643379</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Platform Technician I</t>
+          <t>Multi Skilled Technician</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>BlueVoyant</t>
+          <t>JLL</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Manila, National Capital Region, Philippines</t>
+          <t>Batangas, Calabarzon, Philippines</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>46031</v>
+        <v>46033</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1716,7 +1589,7 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/bluevoyant</t>
+          <t>https://www.linkedin.com/company/jll</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -1735,7 +1608,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>li-4332222982</t>
+          <t>li-4345212547</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1745,27 +1618,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4332222982</t>
+          <t>https://www.linkedin.com/jobs/view/4345212547</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Technical Services Technician</t>
+          <t>Deskside Technician</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Datumstruct Philippines, Inc.</t>
+          <t>Stefanini North America and APAC</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Makati, National Capital Region, Philippines</t>
+          <t>Pasay, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1784,7 +1657,7 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://ph.linkedin.com/company/datumstructph</t>
+          <t>https://br.linkedin.com/company/stefanini-na-apac</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -1803,7 +1676,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>li-4314154195</t>
+          <t>li-4334598816</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1813,27 +1686,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4314154195</t>
+          <t>https://www.linkedin.com/jobs/view/4334598816</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026 Data Center Technician Intern</t>
+          <t>Service Technician Castilla y León</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Amazon Web Services (AWS)</t>
+          <t>Vestas</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Bolinao, Ilocos Region, Philippines</t>
+          <t>Buenavista, Western Visayas, Philippines</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1852,7 +1725,7 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/amazon-web-services</t>
+          <t>https://dk.linkedin.com/company/vestas</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -1871,7 +1744,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>li-4331574126</t>
+          <t>li-4350237071</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1881,27 +1754,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4331574126</t>
+          <t>https://www.linkedin.com/jobs/view/4350237071</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Multi-Skilled Technician - Makati</t>
+          <t>Technician I, Managed Services</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>CBRE Asia Pacific</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Makati, National Capital Region, Philippines</t>
+          <t>Quezon City, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1920,7 +1793,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
+          <t>https://www.linkedin.com/company/copeland</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -1939,7 +1812,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>li-4352057410</t>
+          <t>li-4350286936</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1949,27 +1822,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4352057410</t>
+          <t>https://www.linkedin.com/jobs/view/4350286936</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Associate, Technical Services</t>
+          <t>Technician I, Managed Sevices</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Vena Group</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Ilocos Region, Philippines</t>
+          <t>Quezon City, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1988,7 +1861,7 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://sg.linkedin.com/company/venagroup</t>
+          <t>https://www.linkedin.com/company/copeland</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -2007,7 +1880,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>li-4359761815</t>
+          <t>li-4359757191</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2017,27 +1890,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359761815</t>
+          <t>https://www.linkedin.com/jobs/view/4359757191</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Technician I - Reliability</t>
+          <t>Medewerker Technische Dienst</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Microchip Technology Inc.</t>
+          <t>Stayokay</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Davao, Davao Region, Philippines</t>
+          <t>Bacnotan, Ilocos Region, Philippines</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -2056,7 +1929,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/microchip-technology</t>
+          <t>https://nl.linkedin.com/company/stayokay</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -2075,7 +1948,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>li-4359761816</t>
+          <t>li-4350187030</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2085,27 +1958,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359761816</t>
+          <t>https://www.linkedin.com/jobs/view/4350187030</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Technician I - Reliability</t>
+          <t>Technician I, Managed Services</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Microchip Technology Inc.</t>
+          <t>Copeland</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Davao, Davao Region, Philippines</t>
+          <t>Quezon City, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46031</v>
+        <v>46032</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -2124,7 +1997,7 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/microchip-technology</t>
+          <t>https://www.linkedin.com/company/copeland</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -2143,7 +2016,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>li-4359611660</t>
+          <t>li-4345577544</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2153,28 +2026,26 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359611660</t>
+          <t>https://www.linkedin.com/jobs/view/4345577544</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Multi-Skilled Technician</t>
+          <t>IS Technician - ISHELP</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>JLL</t>
+          <t>GHD</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Makati, National Capital Region, Philippines</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>46031</v>
-      </c>
+          <t>Cebu, Central Visayas, Philippines</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -2192,7 +2063,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/jll</t>
+          <t>https://au.linkedin.com/company/ghd</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -2211,7 +2082,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>li-4358913747</t>
+          <t>li-4351819555</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2221,28 +2092,26 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4358913747</t>
+          <t>https://www.linkedin.com/jobs/view/4351819555</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tech Svc Desk</t>
+          <t>Multi Skilled Technician</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Unisys</t>
+          <t>FPD ASIA PROPERTY SERVICES, INC.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Manila, National Capital Region, Philippines</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>46030</v>
-      </c>
+          <t>Taguig, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
@@ -2260,7 +2129,7 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/unisys</t>
+          <t>https://ph.linkedin.com/company/fpd-asia-property-services-inc-</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2279,7 +2148,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>li-4358576241</t>
+          <t>li-4332549682</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2289,28 +2158,26 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4358576241</t>
+          <t>https://www.linkedin.com/jobs/view/4332549682</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sr Tech Svc Desk</t>
+          <t>Pump Technician</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Unisys</t>
+          <t>Trade One Incorporated</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Manila, National Capital Region, Philippines</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>46030</v>
-      </c>
+          <t>Quezon City, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
@@ -2328,7 +2195,7 @@
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/unisys</t>
+          <t>https://ph.linkedin.com/company/tradeoneincorporated</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2347,7 +2214,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>li-4359757191</t>
+          <t>li-4361161826</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2357,23 +2224,23 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359757191</t>
+          <t>https://www.linkedin.com/jobs/view/4361161826</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Medewerker Technische Dienst</t>
+          <t>Multi-Skilled Technician</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Stayokay</t>
+          <t>CBRE Asia Pacific</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Bacnotan, Ilocos Region, Philippines</t>
+          <t>Lipa, Calabarzon, Philippines</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -2394,7 +2261,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/stayokay</t>
+          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2413,7 +2280,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>li-4359964843</t>
+          <t>li-4354460426</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2423,23 +2290,23 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359964843</t>
+          <t>https://www.linkedin.com/jobs/view/4354460426</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Multi Skilled Technician</t>
+          <t>Multi-Skilled Technician - Lipa</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>JLL</t>
+          <t>CBRE Asia Pacific</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Makati, National Capital Region, Philippines</t>
+          <t>Lipa, Calabarzon, Philippines</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -2460,7 +2327,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/jll</t>
+          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2479,7 +2346,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>li-4345800265</t>
+          <t>li-4345634591</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2489,23 +2356,23 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4345800265</t>
+          <t>https://www.linkedin.com/jobs/view/4345634591</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SRE Technician</t>
+          <t>SAP Academy for Services &amp; Consulting (APAC) - Technical Quality Manager (TQM) - Philippines</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>STMicroelectronics</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Calamba, Northern Mindanao, Philippines</t>
+          <t>Taguig, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -2526,7 +2393,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://ch.linkedin.com/company/stmicroelectronics</t>
+          <t>https://de.linkedin.com/company/sap</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -2542,134 +2409,6 @@
       <c r="AG25" t="inlineStr"/>
       <c r="AH25" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>li-4334726725</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4334726725</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Renewables Technical Lead</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Aggreko</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="b">
-        <v>0</v>
-      </c>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>https://uk.linkedin.com/company/aggreko</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="inlineStr"/>
-      <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
-      <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
-      <c r="AF26" t="inlineStr"/>
-      <c r="AG26" t="inlineStr"/>
-      <c r="AH26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>li-4360643379</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4360643379</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Multi Skilled Technician</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>JLL</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Batangas, Calabarzon, Philippines</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="b">
-        <v>0</v>
-      </c>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/jll</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
-      <c r="AB27" t="inlineStr"/>
-      <c r="AC27" t="inlineStr"/>
-      <c r="AD27" t="inlineStr"/>
-      <c r="AE27" t="inlineStr"/>
-      <c r="AF27" t="inlineStr"/>
-      <c r="AG27" t="inlineStr"/>
-      <c r="AH27" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
adjust html to properly display new jobs for the day
</commit_message>
<xml_diff>
--- a/iTrack/scraped_jobs.xlsx
+++ b/iTrack/scraped_jobs.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH25"/>
+  <dimension ref="A1:AH28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,7 +607,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>in-a0f2177ec4d1d3ea</t>
+          <t>in-24bbb1027ad4d416</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -617,31 +617,31 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://ph.indeed.com/viewjob?jk=a0f2177ec4d1d3ea</t>
+          <t>https://ph.indeed.com/viewjob?jk=24bbb1027ad4d416</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>http://ph.indeed.com/job/accounting-intern-a0f2177ec4d1d3ea</t>
+          <t>https://jobs.lever.co/ninjavan/3ae83fe9-6325-4551-9fea-7a46fe87b508?lever-source=Indeed</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Accounting Intern</t>
+          <t>Human Resources Intern</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Agile Tech Ops Ince</t>
+          <t>Ninja Van</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ayala Avenue-Paseo de Roxas, P00, PH</t>
+          <t>Taguig, P00, PH</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46035</v>
+        <v>46037</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -661,6 +661,661 @@
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
+        <is>
+          <t>Ninja Van is a tech\-enabled logistics company on a mission to provide hassle\-free delivery services for businesses of all sizes across Southeast Asia. Launched in 2014, we started operations in Singapore and have become the region's largest and fastest growing last\-mile logistics company, partnering with over 35,000 merchants and delivering more than 1,000 parcels every minute across six countries.  
+At our core, we are a technology company that is disrupting a massive industry with cutting\-edge software and operational concepts. Powered by algorithm\-based optimisation, dynamic routing, end\-to\-end tracking and a data\-driven approach, we provide best\-of\-class delivery services that delight both the shippers and end customers. But we are just getting started! We have much room for improvement and many ideas that will further shape the industry.  
+The **Human Resources Unit** manages the entire life cycle of each employee \- from attraction, recruitment, onboarding, development, retention and separation. The unit focuses on strategizing initiatives and solutions that build a close\-knit culture, encourages professional and leadership growth and drive high performance among employees. It also ensures that the company is compliant to work and compensation standards set by relevant government agencies such as the Department of Labor.  
+As part of the Human Resources Unit, the **Human Resources Intern** will gain hands\-on exposure across key HR functions, supporting the team in managing the employee life cycle. The intern will be involved in **Talent Acquisition** by assisting with recruitment activities such as candidate screening, interview coordination, job postings, and recruitment reporting. They will also support **Compensation and Benefits** initiatives through administrative assistance in payroll processing, benefits documentation, data tracking, and coordination with internal stakeholders. In **Employee Relations**, the intern will help address employee inquiries, support documentation of HR cases, assist in employee engagement activities, and ensure proper maintenance of employee records in compliance with company policies and labor regulations.
+This role provides a strong foundation for understanding how HR strategies support Ninja Van’s fast\-paced, tech\-enabled logistics operations while contributing to a positive and high\-performing workplace culture.
+Submit a job application
+By applying to the job, you acknowledge that you have read, understood and agreed to our Privacy Policy Notice (the “Notice”) and consent to the collection, use and/or disclosure of your personal data by Ninja Logistics Pte Ltd (the “Company”) for the purposes set out in the Notice. In the event that your job application or personal data was received from any third party pursuant to the purposes set out in the Notice, you warrant that such third party has been duly authorised by you to disclose your personal data to us for the purposes set out in the the Notice.
+We may use artificial intelligence (AI) tools to support parts of the hiring process, such as reviewing applications, analyzing resumes, or assessing responses. These tools assist our recruitment team but do not replace human judgment. Final hiring decisions are ultimately made by humans. If you would like more information about how your data is processed, please contact us.</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/cmp/Ninja-Van</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>https://d2q79iu7y748jz.cloudfront.net/s/_squarelogo/256x256/81bcc11b57b5954b98c86f9d8b8281e7</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>https://www.ninjavan.co/en-sg</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>501 to 1,000</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>$5M to $25M (USD)</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Our Mission: Connecting Southeast Asia to a world of possibilities, one delightful delivery at a time</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>in-86321f8f56c390bb</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/viewjob?jk=86321f8f56c390bb</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/accounting-intern-86321f8f56c390bb</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Accounting Intern</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Circuit Solutions Incorporated</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pasig, P00, PH</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>fulltime, internship</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>*Be part of our EXCITE (Experience CSI Internship in Tech Entrepreneurship) Program!*
+**Qualifications:**
+* Currently taking up Accounting, Financial Management, or Accounting Management
+* Full\-time intern, available to work Monday to Friday
+* Proficient in MS Excel
+* With understanding of basic accounting principles
+* Able to investigate and resolve issues independently
+* High attention to detail and accuracy
+* With positive attitude and strong passion for learning
+* Number of slot available: 1
+Job Types: Full\-time, OJT (On the job training)
+Pay: Php150\.00 \- Php200\.00 per day
+Application Question(s):
+* Do you have other subjects enrolled aside from your OJT?
+* When can you start?
+* How many hours is required for your internship?
+* Are you willing to do on\-site internship?
+Work Location: In person</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/cmp/Circuit-Solutions-Incorporated</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>in-7d475c3a40bef8c0</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/viewjob?jk=7d475c3a40bef8c0</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/ojt-intern-human-resource-hrd-7d475c3a40bef8c0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OJT | Intern Human Resource ( HRD )</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Nutra Tech Biopharma, Inc.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Silang, 04A, PH</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>\- Currently enrolled in a Bachelor’s degree related to Human Resources, Psychology, Business Administration, or equivalent  
+\- location: Balubad, 2nd Silang Cavite  
+\-Required by school to complete an internship or OJT program
+The HR Intern / OJT assists the Human Resources Department in daily administrative and operational tasks while gaining hands\-on experience in HR functions. The role supports recruitment, employee records management, training coordination, and general HR activities in compliance with company policies.
+Job Type: OJT (On the job training)
+Work Location: In person</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/cmp/Nutra-Tech-Biopharma,-Inc.</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>in-409ca859cb1b332c</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/viewjob?jk=409ca859cb1b332c</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/accounting-intern-409ca859cb1b332c</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Accounting Intern</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PBO Global</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Work from Home, PH</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>fulltime, internship</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>**Summary:**
+The objective of the program is to develop students into skilled accounting professionals who can contribute to the finance and accounting team. PBO Global is offering a remote Accounting Internship Program designed to provide practical, hands\-on experience in accounting operations, financial reporting, and business processes. This internship is suitable for students or fresh graduates looking to gain real\-world accounting experience in a corporate environment.
+This program runs for 2 to 4 months in line with the on\-the\-job training requirements of your school or university.
+**Duties \&amp; Responsibilities:**
+* Assisting the accounting team with day\-to\-day financial operations.
+* Recording and reconciling financial transactions using accounting software and MS Excel.
+* Supporting accounts payable and accounts receivable processes.
+* Assisting in preparing financial reports, statements, and summaries.
+* Conducting basic financial analysis and reporting.
+* Maintaining proper documentation and filing of financial records.
+* Supporting budgeting and expense monitoring activities.
+* Learning internal controls and compliance procedures.
+* Recording transactions and reconciling accounts.
+* Assisting with month\-end and year\-end financial closings.
+* Supporting payroll and billing processes.
+* Generating reports for management review.
+* Collaborating with the accounting team on audits and financial reviews.
+* Performing general administrative tasks to support the finance function.
+**Qualifications \&amp; Requirements:**
+* Open to college, vocational, or senior high school graduates interested in gaining practical accounting experience.
+* Enrolled in or graduated from courses related to Accounting, Finance, Business Administration, or ABM strand (for senior high school).
+* Strong numerical and analytical skills.
+* Proficient in MS Office, especially Excel.
+* Basic understanding of accounting principles and financial concepts.
+* Tech\-savvy and comfortable working remotely.
+* Self\-motivated, organized, and able to manage tasks independently.
+Job Types: Full\-time, OJT (On the job training)  
+Contract length: 4 months
+Benefits:
+* Work from home
+Work Location: Remote</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/cmp/Pbo-Global-1</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>https://pboglobal.com.au/</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Clark Center, Unit B 5th Floor Clark Center 7 Berthaphil, Jose Abad Santos Ave, Clark, 2023 Pampanga</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>11 to 50</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>in-e3ef37eb705926ce</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/viewjob?jk=e3ef37eb705926ce</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://ag.wd3.myworkdayjobs.com/en-US/Airbus/job/Pasay-City/Technical-Support-Intern_JR10382626</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Technical Support Intern</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pasay, P00, PH</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>46036</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>emsom@airbus.com</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>**Job Description:**
+**Responsibilities:**
+* Assist in monitoring key performance indicators in the implementation of maintenance projects
+* Assist in the procurement of products, services, and other materials
+* Assosit in the preparation of costing and checking on the availability of data for spare parts and services within Airbus Helicopters Group or from an external supplier
+* Assist in the preparation of quotations under consideration of required maintenance man\-hours and cost for spare parts, materials, and services.
+* Assist in the preparation and issuance of purchase orders
+* Assist in monitoring all the orders and follow up on the undelivered spares from suppliers
+* Encoding of all parts ordered under order monitoring in the database
+* Adherence to company’s rules and regulations and safety policy
+**Personal \&amp; Interpersonal Skills**
+* Meticulous and keen on details
+* Performs job with the highest integrity
+* Promotes camaraderie among employees
+* Good communication skills (written and oral)
+* Tech\-Savvy
+* Knowledge in Aviation Industry is an advantage
+Professional skills:
+* Currently enrolled in Bachelor’s Degree in Aeronautical Engineering or any aviation related\-courses
+This job requires an awareness of any potential compliance risks and a commitment to act with integrity, as the foundation for the Company’s success, reputation and sustainable growth.
+**Company:**
+Airbus Helicopters Philippines Inc.
+**Employment Type:**
+Internship
+\-
+**Experience Level:**
+Student
+**Job Family:**
+Support to Management \&lt;JF\-FA\-ES\&gt;
+By submitting your CV or application you are consenting to Airbus using and storing information about you for monitoring purposes relating to your application or future employment. This information will only be used by Airbus.
+Airbus is committed to achieving workforce diversity and creating an inclusive working environment. We welcome all applications irrespective of social and cultural background, age, gender, disability, sexual orientation or religious belief.
+Airbus is, and always has been, committed to equal opportunities for all. As such, we will never ask for any type of monetary exchange in the frame of a recruitment process. Any impersonation of Airbus to do so should be reported to emsom@airbus.com .
+At Airbus, we support you to work, connect and collaborate more easily and flexibly. Wherever possible, we foster flexible working arrangements to stimulate innovative thinking.</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/cmp/Airbus-e4b213b1</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>https://www.airbus.com</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>10,000+</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>more than $10B (USD)</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>We look to recruit, develop, grow and retain the best, and welcome ALL as an equal opportunity employer.</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>in-46b21c09a7f9b13b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/viewjob?jk=46b21c09a7f9b13b</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/project-management-intern-sports-46b21c09a7f9b13b</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Project Management Intern (Sports)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>XMPLR</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pasig, P00, PH</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>46035</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>**Project Management Intern**
+The project management Intern is responsible for the day\-to\-day management of all aspects of XMPLR projects and works with other stakeholders to ensure their success.
+**Responsibilities—What you'll do:**
+· Assist in proposing, planning and developing potential project ideas.
+· Collaborate with the project team (e.g. organization staff, third\-party personnel, suppliers, and volunteers etc), for project deliverables
+· Implement and monitor project progress and meet deliverables within agreed timelines
+· Assist in stakeholder communication, resolving problems, conflicts and issues in relation to the projects as a customer service point of contact
+· Lead the development of marketing initiatives and communication campaigns for the projects
+· Lead the development and execution of the project marketing plans, content creation and publication
+· Plan, request and administer the budget allocated for the project
+· Prepare various documents (such as progress reports, budget utilization, customer service etc.) for presentations and audit purposes
+· Evaluate project performance across agreed KPIs in agreed timeframes
+**What will make you successful:**
+· Management, Marketing, or Communication undergrad or related field
+· Experience in project management, critical thinking, relationship management
+· Proactive, organized, detail\-oriented and able to manage multiple tasks simultaneously
+· Excellent communication and leadership skills
+· Fluent in English and Filipino
+· Tech and Social\-media savvy
+· Background in sports is a plus
+Job Type: OJT (On the job training)  
+Contract length: 6 months
+Benefits:
+* Flextime
+Work Location: Hybrid remote in Pasig</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/cmp/Xmplr</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>in-a0f2177ec4d1d3ea</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://ph.indeed.com/viewjob?jk=a0f2177ec4d1d3ea</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>http://ph.indeed.com/job/accounting-intern-a0f2177ec4d1d3ea</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Accounting Intern</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Agile Tech Ops Ince</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ayala Avenue-Paseo de Roxas, P00, PH</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>46035</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>internship</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="b">
+        <v>0</v>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
         <is>
           <t>**JOB TITLE:** Accounting Intern
 **COMPANY:** Agile Tech Ops Inc.
@@ -692,568 +1347,10 @@
 Work Location: In person</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/cmp/Agile-Tech-Ops-Ince</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>in-225d4b3b461348b2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/viewjob?jk=225d4b3b461348b2</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://intrepid.bamboohr.com/careers/1521?source=indeed&amp;src=indeed&amp;postedDate=2026-01-11</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Finance Intern (Required Internship Only)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Intrepid</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Manila, P00, PH</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>46033</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>internship</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="b">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>**Who we are**
-Intrepid Asia is a leading Ecommerce and Digital Solutions Provider in South East Asia. We offer end\-to\-end omni\-channel ecommerce management, Livestreaming, Video production \&amp; Affiliate Management for Social Commerce plus full funnel Digital Marketing Services and advanced Market Intelligence, all powered by state of the art inhouse Technology to our client base of leading international brands across all key marketplaces and social platforms in all 6 SEA countries. Brands love our regional presence, our excellent data\-driven and growth\-focused services which are enabled by the strongest team in the industry, and our advanced marketing and tech capabilities.
-We are growing rapidly and as the exclusive partner of Flywheel in SEA, we offer many exciting opportunities to work with leading brands across multiple categories and key industry players. By joining us, you will work on the cutting edge of digital and social commerce in SEA, and experience what it takes to drive a successful ecommerce business end\-to\-end.
- **The team you will be part of**
-Our Finance Team is at the core of every major decision we make. We don’t just keep the books — we shape the direction of the business. By delivering on financial insights, strategic analysis, and data\-driven recommendations, the team plays a critical role in guiding growth and ensuring long\-term success. From planning and forecasting to optimizing performance and supporting key commercial initiatives, Our Finance team is a key partner across every function. With a strong focus on integrity, accuracy, and collaboration, its goal is to ensure the company remains financially strong, agile, and ready for the future.
- **The part you will play**
-We are looking for a Finance Intern who will be an active contributor to our Finance team. This role will report directly to the Senior Accountant and will provide hands\-on exposure to day\-to\-day finance operations, including accounting support, documentation, and financial administrative tasks. You will work closely with the Finance team and gain practical experience in a fast\-paced ecommerce environment.
- **As a Finance Intern, you will take charge of**
-* Assisting in the preparation and issuance of retail sales invoices
-* Filing, organizing, and maintaining accounting and finance documents
-* Supporting liquidation, reimbursement, and expense claims processes
-* Assisting in accounts receivable and accounts payable tracking
-* Helping ensure completeness and accuracy of financial records
-* Supporting month\-end and ad\-hoc finance reporting tasks
-* Coordinating with internal teams regarding finance\-related documentation
-* Performing other administrative and operational finance tasks as assigned
-**What we are looking for \- the ideal profile**
-* Currently pursuing a Bachelor’s degree in Finance, Accounting, Management Accounting, Business Administration, or a related course
-* Internship **must be a required internship** as part of the university curriculum
-* Able to commit for the full required internship period (minimum duration as required by school)
-* Basic understanding of accounting and finance principles
-* Proficient in Microsoft Suite and Google Workspace
-* Strong attention to detail and good organizational skills
-* Able to handle confidential financial information with integrity
-* Willing to learn, proactive, and able to work in a team environment
-**In return, you will be getting**
-* Join an all\-star Finance team which continues to raise the bar, with systems and processes (and company stability) at the level of sophistication of a small multinational, but with a 'start\-up' spirit of innovation and continuous improvement in an ever\-evolving world
-* In terms of learning opportunities, our organization is second to none. You will get to work on a variety of business models across many different clients as if we are 5 companies in one, and everyone is involved in projects to drive further improvement.
-* Regional teams and country Finance teams collaborate closely to ensure all finance aspects of our business are optimized, giving you a wide exposure and enhanced learning curve in a close\-knit and supportive team
-**We also offer**
-**Best of Both Worlds**
-We are a scale up: the sophistication of a small multinational, with the agility of a start\-up. This means you get to work on cutting\-edge projects, and besides your 'standard' job description, we love to see you show entrepreneurial initiative and want to see your take on how you can take your role and our company to the next level. Good ideas get implemented. You are the master of your own destiny.
- **Culture that Brings Out the Best**
-At Intrepid, culture is not just a buzzword, it is what we practice at work every day. We believe in collaboration over competition, transparency over politics, and willingness to learn over ego. You will be part of a team where people genuinely support one another, celebrate wins together, and face challenges head\-on as one. We put our all into the work but we balance it with fun, whether that is through team lunches, after\-work hangouts, events or shared laughter in the office. This is a place where you can thrive professionally while having a great time.
- **Grow Without Limits**
-Learning at Intrepid is constant and dynamic. You will have access to formal training through face\-to\-face sessions, coaching and our very own Intrepid Academy. On top of that, real\-world experience such as leading clients, working with advanced tech, and mastering best\-in\-class processes will accelerate your growth every step of the way. Surrounded by a talented team that raises the bar daily, in a rapidly growing and ever\-expanding business, the opportunities for your development are endless.
- **Rewarding You Right**
-We believe great work deserves great rewards at Intrepid. That’s why we offer competitive compensation and generous benefits, including comprehensive insurance and ample leave, to support you both in and out of the workplace. We want you to feel valued, cared for, and empowered to bring your best self to work every day.
- *Note: We will not be accepting any unsolicited resumes or CVs from headhunting or recruitment agencies at this point. Any CVs or profiles shared with us will not be entertained, and in the event of dispute, Intrepid will not be liable for any material compensation to third parties*</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/cmp/Intrepid-1c14aa57</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>in-2dbb6c5d669cc55a</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/viewjob?jk=2dbb6c5d669cc55a</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://intrepid.bamboohr.com/careers/1520?source=indeed&amp;src=indeed&amp;postedDate=2026-01-11</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Human Resources Intern (Required Internship Only)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Intrepid</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Manila, P00, PH</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>46033</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>internship</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="b">
-        <v>0</v>
-      </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>**Who we are**
-Intrepid Asia is a leading Ecommerce and Digital Solutions Provider in South East Asia. We offer end\-to\-end omni\-channel ecommerce management, Livestreaming, Video production \&amp; Affiliate Management for Social Commerce plus full funnel Digital Marketing Services and advanced Market Intelligence, all powered by state of the art inhouse Technology to our client base of leading international brands across all key marketplaces and social platforms in all 6 SEA countries. Brands love our regional presence, our excellent data\-driven and growth\-focused services which are enabled by the strongest team in the industry, and our advanced marketing and tech capabilities.
-We are growing rapidly and as the exclusive partner of Flywheel in SEA, we offer many exciting opportunities to work with leading brands across multiple categories and key industry players. By joining us, you will work on the cutting edge of digital and social commerce in SEA, and experience what it takes to drive a successful ecommerce business end\-to\-end.
- **The team you will be part of**
-Our Talent \&amp; People Team is the heartbeat of our organization \- championing a culture where people thrive and potential is unlocked. From attracting top talent and shaping employee experiences to driving development, engagement, and retention, the team plays a strategic role in building and maintaining a high\-performing, empowered workforce. We are here to grow with the business and for the people behind it.
- **The part you will play**
-We are looking for a Human Resources Intern who will be an active contributor to our People Operations team. This role will report directly to our People Operations Specialist and will provide hands\-on exposure to various HR functions, supporting daily operations and ongoing initiatives.
- **As an HR Intern, you will take charge of**
-* Assisting in preparing orientation materials and schedules for new employees
-* Helping maintain employee records and ensure confidentiality
-* Supporting the resolution of employee queries and concerns
-* Assisting in organizing employee engagement activities and events
-* Assisting in maintaining and updating HR 201 files and database
-* Assisting in the preparation of HR\-related reports and documents as needed
-* Assisting in coordinating training sessions and workshops
-* Participating in the development of training materials
-* Providing general administrative support to the HR department
-* Participating in HR projects and initiatives as assigned
-**What we are looking for \- the ideal profile**
-* Currently pursuing a degree in Human Resource Management, Psychology, or other related fields, **with an internship requirement**
-* Strong written and verbal communication skills
-* Proficient in MS Office applications and Google Workspace
-* Detail\-oriented with the ability to handle sensitive and confidential information
-* Strong organizational skills with the ability to manage multiple tasks and meet deadlines
-**In return, you will be getting**
-* Tackling the sophisticated people's challenges in the rapidly evolving e\-commerce landscape with data insights and innovative solutions.
-* You will be joining an all\-star People Team that consistently raises the bar by combining the systems and processes of a small multinational with the collaborative, innovative, and agile spirit of a startup in an ever\-evolving world.
-* With our team’s rapid growth and the People Team launching new initiatives to enhance both employee experience and performance, you will benefit from a wide range of opportunities for development. Our structured learning programs covering both functional skills and broader growth are designed to support you at every stage of your journey
-* Our supportive culture and close collaboration between regional and local teams create a close\-knit work environment which many in our team love and thrive in
-**We also offer**
-**Best of Both Worlds**
-We are a scale up: the sophistication of a small multinational, with the agility of a start\-up. This means you get to work on cutting\-edge projects, and besides your 'standard' job description, we love to see you show entrepreneurial initiative and want to see your take on how you can take your role and our company to the next level. Good ideas get implemented. You are the master of your own destiny.
- **Culture that Brings Out the Best**
-At Intrepid, culture is not just a buzzword, it is what we practice at work every day. We believe in collaboration over competition, transparency over politics, and willingness to learn over ego. You will be part of a team where people genuinely support one another, celebrate wins together, and face challenges head\-on as one. We put our all into the work but we balance it with fun, whether that is through team lunches, after\-work hangouts, events or shared laughter in the office. This is a place where you can thrive professionally while having a great time.
- **Grow Without Limits**
-Learning at Intrepid is constant and dynamic. You will have access to formal training through face\-to\-face sessions, coaching and our very own Intrepid Academy. On top of that, real\-world experience such as leading clients, working with advanced tech, and mastering best\-in\-class processes will accelerate your growth every step of the way. Surrounded by a talented team that raises the bar daily, in a rapidly growing and ever\-expanding business, the opportunities for your development are endless.
- **Rewarding You Right**
-We believe great work deserves great rewards at Intrepid. That’s why we offer competitive compensation and generous benefits, including comprehensive insurance and ample leave, to support you both in and out of the workplace. We want you to feel valued, cared for, and empowered to bring your best self to work every day.
- *Note: We will not be accepting any unsolicited resumes or CVs from headhunting or recruitment agencies at this point. Any CVs or profiles shared with us will not be entertained, and in the event of dispute, Intrepid will not be liable for any material compensation to third parties*</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/cmp/Intrepid-1c14aa57</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>in-f1e13e490a93b540</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/viewjob?jk=f1e13e490a93b540</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>http://ph.indeed.com/job/it-programming-intern-f1e13e490a93b540</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>IT / Programming Intern</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Lucky Boba</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Sangandaan, P00, PH</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>46032</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>temporary, internship</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="b">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>luckyboba.hr@gmail.com</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>**We're Hiring Interns!**
-Are you passionate about technology and eager to gain  
-hands\-on experience in IT and programming? Join our team and kickstart your  
-career!
-**Position:** IT / Programming Intern
-**Who We’re Looking For:**  
-**Students currently pursuing:**
-IT Programming  
-Computer Engineering  
-Computer Science  
-Any Programming\-related course
-**What You’ll Do:**  
-Assist in software development and coding projects  
-Support IT operations and system maintenance  
-Collaborate with our tech team on real\-world projects  
-Learn best practices in programming, debugging, and testing
-**What We’re Looking For:**  
-Strong interest in programming and technology  
-Basic knowledge of programming languages (e.g., Java, Python, C\#, or JavaScript)  
-Eagerness to learn and take on challenges  
-Good communication and teamwork skills
-**Perks \&amp; Benefits:**  
-Hands\-on experience in real projects  
-Mentorship from experienced developers  
-Flexible working hours  
-Certificate of Internship upon completion
-**How to Apply:**  
-Submit your CV \&amp; Portfolio**: luckyboba.hr@gmail.com**
-Start your tech journey with us!
-Job Types: Temporary, OJT (On the job training)  
-Contract length: 3 months
-Benefits:
-* Flexible schedule
-* Flextime
-Work Location: In person</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>https://ph.indeed.com/cmp/Lucky-Boba-1</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>li-4332535951</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4332535951</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Technician 1 Monitoring Services (Technical Support)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Risewave Consulting, Inc.</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>https://ph.linkedin.com/company/risewave-consulting-inc</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>li-4359997663</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4359997663</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Multi Skilled Technician (Taguig)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>JLL</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Taguig, National Capital Region, Philippines</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="b">
-        <v>0</v>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/company/jll</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>li-4352672394</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>https://www.linkedin.com/jobs/view/4352672394</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PHL Senior Technician - L3 - Represented/Tariff</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Dow</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Las Piñas, National Capital Region, Philippines</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>46034</v>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="b">
-        <v>0</v>
-      </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/dow-chemical</t>
+          <t>https://ph.indeed.com/cmp/Agile-Tech-Ops-Ince</t>
         </is>
       </c>
       <c r="W8" t="inlineStr"/>
@@ -1272,7 +1369,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>li-4351866176</t>
+          <t>li-4355150222</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1282,27 +1379,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4351866176</t>
+          <t>https://www.linkedin.com/jobs/view/4355150222</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Multi-Skilled Technician -Lipa</t>
+          <t>NAPA Technician</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CBRE Asia Pacific</t>
+          <t>Ng Khai Development Corporation</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Lipa, Calabarzon, Philippines</t>
+          <t>Cebu, Central Visayas, Philippines</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>46034</v>
+        <v>46036</v>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -1321,7 +1418,7 @@
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
-          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
+          <t>https://ph.linkedin.com/company/ng-khai-development-corporation</t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
@@ -1340,7 +1437,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>li-4345396142</t>
+          <t>li-4355110581</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1350,27 +1447,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4345396142</t>
+          <t>https://www.linkedin.com/jobs/view/4355110581</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Multi-Skilled Technician - Lipa</t>
+          <t>Multi Skilled Technician</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CBRE Asia Pacific</t>
+          <t>FPD ASIA PROPERTY SERVICES, INC.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lipa, Calabarzon, Philippines</t>
+          <t>Taguig, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>46034</v>
+        <v>46036</v>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1389,7 +1486,7 @@
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
+          <t>https://ph.linkedin.com/company/fpd-asia-property-services-inc-</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
@@ -1408,7 +1505,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>li-4334726725</t>
+          <t>li-4346096853</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1418,23 +1515,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4334726725</t>
+          <t>https://www.linkedin.com/jobs/view/4346096853</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Renewables Technical Lead</t>
+          <t>SERVICE TECHNICIAN (SAN PEDRO OFFICE BASED)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Aggreko</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>EPTA GROUP</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Muntinlupa City, National Capital Region, Philippines</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="n">
-        <v>46033</v>
+        <v>46036</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1453,7 +1554,7 @@
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>https://uk.linkedin.com/company/aggreko</t>
+          <t>https://it.linkedin.com/company/epta-group</t>
         </is>
       </c>
       <c r="W11" t="inlineStr"/>
@@ -1472,7 +1573,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>li-4359964843</t>
+          <t>li-4355013135</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1482,27 +1583,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359964843</t>
+          <t>https://www.linkedin.com/jobs/view/4355013135</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Multi Skilled Technician</t>
+          <t>Multi - Skilled Technician</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>JLL</t>
+          <t>Med-Metrix</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Makati, National Capital Region, Philippines</t>
+          <t>Pasig, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>46033</v>
+        <v>46036</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1521,7 +1622,7 @@
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/jll</t>
+          <t>https://www.linkedin.com/company/med-metrix</t>
         </is>
       </c>
       <c r="W12" t="inlineStr"/>
@@ -1540,7 +1641,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>li-4360643379</t>
+          <t>li-4354868085</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1550,27 +1651,23 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4360643379</t>
+          <t>https://www.linkedin.com/jobs/view/4354868085</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Multi Skilled Technician</t>
+          <t>Technical Lead (Senior Full Stack)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>JLL</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Batangas, Calabarzon, Philippines</t>
-        </is>
-      </c>
+          <t>Mediatropy</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" s="2" t="n">
-        <v>46033</v>
+        <v>46036</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1589,7 +1686,7 @@
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/jll</t>
+          <t>https://sg.linkedin.com/company/mediatropy</t>
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
@@ -1608,7 +1705,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>li-4345212547</t>
+          <t>li-4354705043</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1618,27 +1715,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4345212547</t>
+          <t>https://www.linkedin.com/jobs/view/4354705043</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Deskside Technician</t>
+          <t>STP Technician</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Stefanini North America and APAC</t>
+          <t>Metro Pacific Water Solutions, Inc.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pasay, National Capital Region, Philippines</t>
+          <t>Davao, Davao Region, Philippines</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>46032</v>
+        <v>46035</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1657,7 +1754,7 @@
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="inlineStr">
         <is>
-          <t>https://br.linkedin.com/company/stefanini-na-apac</t>
+          <t>https://ph.linkedin.com/company/metro-pacific-water-solutions</t>
         </is>
       </c>
       <c r="W14" t="inlineStr"/>
@@ -1676,7 +1773,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>li-4334598816</t>
+          <t>li-4361169891</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1686,27 +1783,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4334598816</t>
+          <t>https://www.linkedin.com/jobs/view/4361169891</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Service Technician Castilla y León</t>
+          <t>Sr Tech Svc Desk</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Vestas</t>
+          <t>Unisys</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Buenavista, Western Visayas, Philippines</t>
+          <t>Manila, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>46032</v>
+        <v>46035</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1725,7 +1822,7 @@
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/company/vestas</t>
+          <t>https://www.linkedin.com/company/unisys</t>
         </is>
       </c>
       <c r="W15" t="inlineStr"/>
@@ -1744,7 +1841,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>li-4350237071</t>
+          <t>li-4308923917</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1754,27 +1851,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4350237071</t>
+          <t>https://www.linkedin.com/jobs/view/4308923917</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Technician I, Managed Services</t>
+          <t>Technician III</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>Microchip Technology Inc.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
+          <t>Davao, Davao Region, Philippines</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>46032</v>
+        <v>46035</v>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1793,7 +1890,7 @@
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/copeland</t>
+          <t>https://www.linkedin.com/company/microchip-technology</t>
         </is>
       </c>
       <c r="W16" t="inlineStr"/>
@@ -1812,7 +1909,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>li-4350286936</t>
+          <t>li-4354495027</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1822,27 +1919,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4350286936</t>
+          <t>https://www.linkedin.com/jobs/view/4354495027</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Technician I, Managed Sevices</t>
+          <t>Mega FM Technician, SPX Express (Zone 1 - Parañaque / Las Piñas)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>SPX Express</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
+          <t>Manila, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>46032</v>
+        <v>46035</v>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1861,7 +1958,7 @@
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/copeland</t>
+          <t>https://www.linkedin.com/company/spx-express</t>
         </is>
       </c>
       <c r="W17" t="inlineStr"/>
@@ -1880,7 +1977,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>li-4359757191</t>
+          <t>li-4340379368</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1890,27 +1987,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4359757191</t>
+          <t>https://www.linkedin.com/jobs/view/4340379368</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Medewerker Technische Dienst</t>
+          <t>Motorpool Service Technician/Mechanical Technician</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Stayokay</t>
+          <t>Aboitiz Foods</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Bacnotan, Ilocos Region, Philippines</t>
+          <t>Iligan, Northern Mindanao, Philippines</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46032</v>
+        <v>46035</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1929,7 +2026,7 @@
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/company/stayokay</t>
+          <t>https://ph.linkedin.com/company/aboitiz-foods</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -1948,7 +2045,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>li-4350187030</t>
+          <t>li-4354460426</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1958,27 +2055,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4350187030</t>
+          <t>https://www.linkedin.com/jobs/view/4354460426</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Technician I, Managed Services</t>
+          <t>Multi-Skilled Technician - Lipa</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Copeland</t>
+          <t>CBRE Asia Pacific</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
+          <t>Lipa, Calabarzon, Philippines</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>46032</v>
+        <v>46034</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1997,7 +2094,7 @@
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/company/copeland</t>
+          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
         </is>
       </c>
       <c r="W19" t="inlineStr"/>
@@ -2016,7 +2113,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>li-4345577544</t>
+          <t>li-4325695361</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2026,23 +2123,23 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4345577544</t>
+          <t>https://www.linkedin.com/jobs/view/4325695361</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>IS Technician - ISHELP</t>
+          <t>Technology - Infrastructure, Summer Analyst (Internship), Philippines, 2026</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>GHD</t>
+          <t>Citi</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Cebu, Central Visayas, Philippines</t>
+          <t>Taguig, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -2063,7 +2160,7 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>https://au.linkedin.com/company/ghd</t>
+          <t>https://www.linkedin.com/company/citi</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>
@@ -2082,7 +2179,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>li-4351819555</t>
+          <t>li-4359145289</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2092,23 +2189,23 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4351819555</t>
+          <t>https://www.linkedin.com/jobs/view/4359145289</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Multi Skilled Technician</t>
+          <t>Field Service/Biomed Technician</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>FPD ASIA PROPERTY SERVICES, INC.</t>
+          <t>OMNIBUS BIO-MEDICAL SYSTEMS INC.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Taguig, National Capital Region, Philippines</t>
+          <t>Hinatuan, Caraga, Philippines</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -2129,7 +2226,7 @@
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
-          <t>https://ph.linkedin.com/company/fpd-asia-property-services-inc-</t>
+          <t>https://ph.linkedin.com/company/omnibus-bio-medical-systems-incorporated</t>
         </is>
       </c>
       <c r="W21" t="inlineStr"/>
@@ -2148,7 +2245,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>li-4332549682</t>
+          <t>li-4359003442</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2158,25 +2255,21 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4332549682</t>
+          <t>https://www.linkedin.com/jobs/view/4359003442</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Pump Technician</t>
+          <t>VIP Gulfstream Technician</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Trade One Incorporated</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Quezon City, National Capital Region, Philippines</t>
-        </is>
-      </c>
+          <t>AEXTECH</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -2195,7 +2288,7 @@
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
-          <t>https://ph.linkedin.com/company/tradeoneincorporated</t>
+          <t>https://ph.linkedin.com/company/aextech</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2214,7 +2307,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>li-4361161826</t>
+          <t>li-4357623505</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2224,23 +2317,23 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4361161826</t>
+          <t>https://www.linkedin.com/jobs/view/4357623505</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Multi-Skilled Technician</t>
+          <t>IS Technician - ISHELP Americas</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CBRE Asia Pacific</t>
+          <t>GHD</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Lipa, Calabarzon, Philippines</t>
+          <t>Cebu, Central Visayas, Philippines</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -2261,7 +2354,7 @@
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
-          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
+          <t>https://au.linkedin.com/company/ghd</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2280,7 +2373,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>li-4354460426</t>
+          <t>li-4359104125</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2290,25 +2383,21 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4354460426</t>
+          <t>https://www.linkedin.com/jobs/view/4359104125</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Multi-Skilled Technician - Lipa</t>
+          <t>Salesforce Technical Lead (Work from home)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CBRE Asia Pacific</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Lipa, Calabarzon, Philippines</t>
-        </is>
-      </c>
+          <t>Application House</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -2317,7 +2406,7 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
       <c r="O24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
@@ -2327,7 +2416,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>https://sg.linkedin.com/company/cbre-asia-pacific</t>
+          <t>https://uk.linkedin.com/company/application-house</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2346,7 +2435,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>li-4345634591</t>
+          <t>li-4357607586</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2356,23 +2445,23 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4345634591</t>
+          <t>https://www.linkedin.com/jobs/view/4357607586</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>SAP Academy for Services &amp; Consulting (APAC) - Technical Quality Manager (TQM) - Philippines</t>
+          <t>Pump Technician</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Trade One Incorporated</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Taguig, National Capital Region, Philippines</t>
+          <t>Quezon City, National Capital Region, Philippines</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -2393,7 +2482,7 @@
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/company/sap</t>
+          <t>https://ph.linkedin.com/company/tradeoneincorporated</t>
         </is>
       </c>
       <c r="W25" t="inlineStr"/>
@@ -2409,6 +2498,204 @@
       <c r="AG25" t="inlineStr"/>
       <c r="AH25" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>li-4362701531</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4362701531</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Senior Technician, Probe PMEE</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Allegro MicroSystems</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="b">
+        <v>0</v>
+      </c>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/allegro-microsystems</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>li-4348356368</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4348356368</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Technician 3, Engineering Services</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Analog Devices</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Cavite, Calabarzon, Philippines</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="b">
+        <v>0</v>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/analog-devices</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>li-4359024458</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4359024458</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Senior Software, Platform, or Product Engineer (Technical Lead)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PCI Tech Center</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Manila, National Capital Region, Philippines</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="b">
+        <v>0</v>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>https://ph.linkedin.com/company/pcitechcenter</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>